<commit_message>
add checks to remove double printing of schedule links
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -44,46 +44,22 @@
     <t xml:space="preserve">keycard_drop_rooms</t>
   </si>
   <si>
+    <t xml:space="preserve">Keydrops today: 1615, 515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1713</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1615</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 814, 1713</t>
+  </si>
+  <si>
     <t xml:space="preserve">Keydrops today: 716</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: 1713</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1615</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 513</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1615, 513</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 716, 515</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814, 515</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1713, 513</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 716, 1615</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1713, 515</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814, 716</t>
-  </si>
-  <si>
     <t xml:space="preserve">Keydrops today: 814</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 716, 513, 515</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814, 513</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -496,7 +472,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45870</v>
+        <v>45901</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>0</v>
@@ -505,22 +481,22 @@
         <v>0</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>10</v>
@@ -528,7 +504,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45871</v>
+        <v>45902</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -548,27 +524,25 @@
         <v>0</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>11</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J3" s="1"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45872</v>
+        <v>45903</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>0</v>
@@ -583,19 +557,15 @@
         <v>100</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45873</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45904</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
       <c r="D5" s="1" t="n">
         <v>0</v>
       </c>
@@ -603,7 +573,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>0</v>
@@ -612,23 +582,25 @@
         <v>0</v>
       </c>
       <c r="I5" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>13</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J5" s="1"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45874</v>
-      </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
+        <v>45905</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="D6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>0</v>
@@ -640,13 +612,15 @@
         <v>0</v>
       </c>
       <c r="I6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45875</v>
+        <v>45906</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -672,7 +646,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45876</v>
+        <v>45907</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -698,22 +672,22 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45877</v>
+        <v>45908</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>0</v>
@@ -725,24 +699,24 @@
         <v>200</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45878</v>
+        <v>45909</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>0</v>
@@ -754,22 +728,20 @@
         <v>0</v>
       </c>
       <c r="I10" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45879</v>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45910</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
       <c r="D11" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>0</v>
@@ -778,26 +750,28 @@
         <v>0</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="H11" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="1" t="n">
-        <v>200</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>15</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J11" s="1"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>45880</v>
-      </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+        <v>45911</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="D12" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
@@ -812,16 +786,22 @@
         <v>0</v>
       </c>
       <c r="I12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>45881</v>
-      </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+        <v>45912</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>1000</v>
+      </c>
       <c r="D13" s="1" t="n">
         <v>0</v>
       </c>
@@ -838,28 +818,26 @@
         <v>0</v>
       </c>
       <c r="I13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>45882</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45913</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
       <c r="D14" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>0</v>
@@ -868,41 +846,45 @@
         <v>0</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>200</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J14" s="1"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>45883</v>
-      </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
+        <v>45914</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="D15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="1"/>
+        <v>200</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>45884</v>
+        <v>45915</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>1000</v>
@@ -920,21 +902,19 @@
         <v>0</v>
       </c>
       <c r="G16" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="H16" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I16" s="1" t="n">
-        <v>200</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>16</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J16" s="1"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>45885</v>
+        <v>45916</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -960,14 +940,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>45886</v>
-      </c>
-      <c r="B18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="1" t="n">
-        <v>1000</v>
-      </c>
+        <v>45917</v>
+      </c>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
       <c r="D18" s="1" t="n">
         <v>0</v>
       </c>
@@ -975,7 +951,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>0</v>
@@ -984,27 +960,21 @@
         <v>0</v>
       </c>
       <c r="I18" s="1" t="n">
-        <v>200</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>17</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J18" s="1"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>45887</v>
-      </c>
-      <c r="B19" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45918</v>
+      </c>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
       <c r="D19" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F19" s="1" t="n">
         <v>0</v>
@@ -1016,23 +986,25 @@
         <v>0</v>
       </c>
       <c r="I19" s="1" t="n">
-        <v>200</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J19" s="1"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>45888</v>
-      </c>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
+        <v>45919</v>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="D20" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>0</v>
@@ -1044,13 +1016,15 @@
         <v>0</v>
       </c>
       <c r="I20" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>45889</v>
+        <v>45920</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1076,13 +1050,13 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>45890</v>
+        <v>45921</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="C22" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="D22" s="1" t="n">
         <v>0</v>
@@ -1094,30 +1068,26 @@
         <v>0</v>
       </c>
       <c r="G22" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="H22" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I22" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>45891</v>
-      </c>
-      <c r="B23" s="1" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C23" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45922</v>
+      </c>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
       <c r="D23" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E23" s="1" t="n">
         <v>0</v>
@@ -1132,22 +1102,18 @@
         <v>0</v>
       </c>
       <c r="I23" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>45892</v>
-      </c>
-      <c r="B24" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C24" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45923</v>
+      </c>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
       <c r="D24" s="1" t="n">
         <v>0</v>
       </c>
@@ -1155,7 +1121,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="G24" s="1" t="n">
         <v>0</v>
@@ -1164,22 +1130,16 @@
         <v>0</v>
       </c>
       <c r="I24" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>13</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J24" s="1"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>45893</v>
-      </c>
-      <c r="B25" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="1" t="n">
-        <v>1000</v>
-      </c>
+        <v>45924</v>
+      </c>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
       <c r="D25" s="1" t="n">
         <v>0</v>
       </c>
@@ -1204,14 +1164,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>45894</v>
-      </c>
-      <c r="B26" s="1" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C26" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45925</v>
+      </c>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
       <c r="D26" s="1" t="n">
         <v>0</v>
       </c>
@@ -1228,27 +1184,21 @@
         <v>0</v>
       </c>
       <c r="I26" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>21</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J26" s="1"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>45895</v>
-      </c>
-      <c r="B27" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45926</v>
+      </c>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
       <c r="D27" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F27" s="1" t="n">
         <v>0</v>
@@ -1260,15 +1210,13 @@
         <v>0</v>
       </c>
       <c r="I27" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J27" s="1"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>45896</v>
+        <v>45927</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>0</v>
@@ -1277,35 +1225,39 @@
         <v>0</v>
       </c>
       <c r="D28" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E28" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F28" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="G28" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="H28" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I28" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>45897</v>
-      </c>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
+        <v>45928</v>
+      </c>
+      <c r="B29" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="D29" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E29" s="1" t="n">
         <v>0</v>
@@ -1326,10 +1278,14 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>45898</v>
-      </c>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
+        <v>45929</v>
+      </c>
+      <c r="B30" s="1" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C30" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="D30" s="1" t="n">
         <v>0</v>
       </c>
@@ -1346,20 +1302,18 @@
         <v>0</v>
       </c>
       <c r="I30" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>45899</v>
-      </c>
-      <c r="B31" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" s="1" t="n">
-        <v>1000</v>
-      </c>
+        <v>45930</v>
+      </c>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
       <c r="D31" s="1" t="n">
         <v>0</v>
       </c>
@@ -1376,67 +1330,33 @@
         <v>0</v>
       </c>
       <c r="I31" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>11</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J31" s="1"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>45900</v>
-      </c>
-      <c r="B32" s="1" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C32" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" s="1" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G32" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="1" t="n">
-        <v>200</v>
-      </c>
-      <c r="J32" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B33" s="3" t="str">
-        <f>SUM(B2:F32)</f>
-      </c>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3" t="str">
-        <f>SUM(G2:H32)</f>
-      </c>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3" t="str">
-        <f>SUM(I2:I32)</f>
+      <c r="A32" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" s="3" t="str">
+        <f>SUM(B2:F31)</f>
+      </c>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3" t="str">
+        <f>SUM(G2:H31)</f>
+      </c>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3" t="str">
+        <f>SUM(I2:I31)</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="G32:H32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
change payments to 1200 after aug 31
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -536,7 +536,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>0</v>
@@ -600,7 +600,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>0</v>
@@ -678,7 +678,7 @@
         <v>0</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>0</v>
@@ -716,7 +716,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>0</v>
@@ -771,7 +771,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
@@ -800,7 +800,7 @@
         <v>0</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="D13" s="1" t="n">
         <v>0</v>
@@ -864,13 +864,13 @@
         <v>0</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="F15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="H15" s="1" t="n">
         <v>0</v>
@@ -887,7 +887,7 @@
         <v>45915</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>0</v>
@@ -1004,7 +1004,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>0</v>
@@ -1053,7 +1053,7 @@
         <v>45921</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>0</v>
@@ -1228,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="E28" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="F28" s="1" t="n">
         <v>0</v>
@@ -1257,7 +1257,7 @@
         <v>0</v>
       </c>
       <c r="D29" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="E29" s="1" t="n">
         <v>0</v>
@@ -1281,7 +1281,7 @@
         <v>45929</v>
       </c>
       <c r="B30" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="C30" s="1" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
start financial statemnts projct
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -44,22 +44,34 @@
     <t xml:space="preserve">keycard_drop_rooms</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: 1615, 515</t>
+    <t xml:space="preserve">Keydrops today: 515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1615</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 513, 515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 513</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 716</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 1713</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: 1615</t>
+    <t xml:space="preserve">Keydrops today: 1713, 716</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 814, 1713, 513</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 814, 1713</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 716</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -472,7 +484,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45901</v>
+        <v>45962</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>0</v>
@@ -484,19 +496,19 @@
         <v>0</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="H2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>10</v>
@@ -504,15 +516,19 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45902</v>
-      </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
+        <v>45963</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="D3" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>0</v>
@@ -524,19 +540,21 @@
         <v>0</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45903</v>
+        <v>45964</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>0</v>
@@ -551,21 +569,25 @@
         <v>0</v>
       </c>
       <c r="H4" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I4" s="1" t="n">
         <v>100</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45904</v>
-      </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
+        <v>45965</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>1200</v>
+      </c>
       <c r="D5" s="1" t="n">
         <v>0</v>
       </c>
@@ -573,34 +595,32 @@
         <v>0</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="1"/>
+        <v>200</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45905</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45966</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
       <c r="D6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>0</v>
@@ -612,15 +632,13 @@
         <v>0</v>
       </c>
       <c r="I6" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J6" s="1"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45906</v>
+        <v>45967</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -646,7 +664,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45907</v>
+        <v>45968</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -666,22 +684,24 @@
         <v>0</v>
       </c>
       <c r="I8" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45908</v>
+        <v>45969</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
@@ -696,27 +716,23 @@
         <v>0</v>
       </c>
       <c r="I9" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45909</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45970</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
       <c r="D10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>0</v>
@@ -728,15 +744,13 @@
         <v>0</v>
       </c>
       <c r="I10" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J10" s="1"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45910</v>
+        <v>45971</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -762,7 +776,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>45911</v>
+        <v>45972</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0</v>
@@ -771,7 +785,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>0</v>
@@ -783,25 +797,21 @@
         <v>0</v>
       </c>
       <c r="H12" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I12" s="1" t="n">
         <v>100</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>45912</v>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="1" t="n">
-        <v>1200</v>
-      </c>
+        <v>45973</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
       <c r="D13" s="1" t="n">
         <v>0</v>
       </c>
@@ -818,26 +828,28 @@
         <v>0</v>
       </c>
       <c r="I13" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>11</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J13" s="1"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>45913</v>
-      </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
+        <v>45974</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="D14" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>0</v>
@@ -846,48 +858,46 @@
         <v>0</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>45914</v>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45975</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
       <c r="D15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>45915</v>
+        <v>45976</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C16" s="1" t="n">
         <v>0</v>
@@ -896,7 +906,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F16" s="1" t="n">
         <v>0</v>
@@ -908,16 +918,22 @@
         <v>0</v>
       </c>
       <c r="I16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>45916</v>
-      </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+        <v>45977</v>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>1200</v>
+      </c>
       <c r="D17" s="1" t="n">
         <v>0</v>
       </c>
@@ -934,13 +950,15 @@
         <v>0</v>
       </c>
       <c r="I17" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>45917</v>
+        <v>45978</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -966,7 +984,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>45918</v>
+        <v>45979</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -992,19 +1010,19 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>45919</v>
+        <v>45980</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C20" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>0</v>
@@ -1016,15 +1034,15 @@
         <v>0</v>
       </c>
       <c r="I20" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>45920</v>
+        <v>45981</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1050,14 +1068,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>45921</v>
-      </c>
-      <c r="B22" s="1" t="n">
-        <v>1200</v>
-      </c>
-      <c r="C22" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45982</v>
+      </c>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
       <c r="D22" s="1" t="n">
         <v>0</v>
       </c>
@@ -1074,15 +1088,13 @@
         <v>0</v>
       </c>
       <c r="I22" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>15</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J22" s="1"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>45922</v>
+        <v>45983</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1102,23 +1114,25 @@
         <v>0</v>
       </c>
       <c r="I23" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J23" s="1"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>45923</v>
-      </c>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
+        <v>45984</v>
+      </c>
+      <c r="B24" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="D24" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F24" s="1" t="n">
         <v>0</v>
@@ -1127,19 +1141,25 @@
         <v>0</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I24" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>45924</v>
-      </c>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
+        <v>45985</v>
+      </c>
+      <c r="B25" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C25" s="1" t="n">
+        <v>1200</v>
+      </c>
       <c r="D25" s="1" t="n">
         <v>0</v>
       </c>
@@ -1147,7 +1167,7 @@
         <v>0</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G25" s="1" t="n">
         <v>0</v>
@@ -1156,15 +1176,15 @@
         <v>0</v>
       </c>
       <c r="I25" s="1" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>45925</v>
+        <v>45986</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1190,7 +1210,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>45926</v>
+        <v>45987</v>
       </c>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1210,25 +1230,23 @@
         <v>0</v>
       </c>
       <c r="I27" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>45927</v>
-      </c>
-      <c r="B28" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45988</v>
+      </c>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
       <c r="D28" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F28" s="1" t="n">
         <v>0</v>
@@ -1240,24 +1258,18 @@
         <v>0</v>
       </c>
       <c r="I28" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J28" s="1"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>45928</v>
-      </c>
-      <c r="B29" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C29" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45989</v>
+      </c>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
       <c r="D29" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E29" s="1" t="n">
         <v>0</v>
@@ -1278,13 +1290,13 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>45929</v>
+        <v>45990</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>1200</v>
       </c>
       <c r="C30" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="D30" s="1" t="n">
         <v>0</v>
@@ -1302,26 +1314,30 @@
         <v>0</v>
       </c>
       <c r="I30" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>45930</v>
-      </c>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
+        <v>45991</v>
+      </c>
+      <c r="B31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="D31" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E31" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F31" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G31" s="1" t="n">
         <v>0</v>
@@ -1330,13 +1346,15 @@
         <v>0</v>
       </c>
       <c r="I31" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B32" s="3" t="str">
         <f>SUM(B2:F31)</f>

</xml_diff>

<commit_message>
switch to manual addjustments for forwarded emails
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,11 +12,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t xml:space="preserve">date</t>
   </si>
   <si>
+    <t xml:space="preserve">310</t>
+  </si>
+  <si>
     <t xml:space="preserve">814</t>
   </si>
   <si>
@@ -60,6 +63,12 @@
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 716</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 310</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1615, 1600</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 1713</t>
@@ -481,6 +490,9 @@
       <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="4" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -502,16 +514,19 @@
         <v>0</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="J2" s="1" t="s">
-        <v>10</v>
+      <c r="K2" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -528,10 +543,10 @@
         <v>0</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>0</v>
@@ -540,10 +555,13 @@
         <v>0</v>
       </c>
       <c r="I3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>11</v>
+      <c r="K3" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -569,13 +587,16 @@
         <v>0</v>
       </c>
       <c r="H4" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I4" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="J4" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>12</v>
+      <c r="K4" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -586,28 +607,31 @@
         <v>0</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>1200</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1" t="n">
         <v>200</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>13</v>
+      <c r="K5" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -616,9 +640,7 @@
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
-      <c r="D6" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D6" s="1"/>
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
@@ -634,7 +656,10 @@
       <c r="I6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="1"/>
+      <c r="J6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="1"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -642,9 +667,7 @@
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
-      <c r="D7" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D7" s="1"/>
       <c r="E7" s="1" t="n">
         <v>0</v>
       </c>
@@ -660,7 +683,10 @@
       <c r="I7" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="1"/>
+      <c r="J7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="1"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -668,9 +694,7 @@
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D8" s="1"/>
       <c r="E8" s="1" t="n">
         <v>0</v>
       </c>
@@ -684,10 +708,13 @@
         <v>0</v>
       </c>
       <c r="I8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>14</v>
+      <c r="K8" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -701,10 +728,10 @@
         <v>0</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>0</v>
@@ -716,10 +743,13 @@
         <v>0</v>
       </c>
       <c r="I9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="J9" s="1" t="s">
-        <v>15</v>
+      <c r="K9" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -728,9 +758,7 @@
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
-      <c r="D10" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D10" s="1"/>
       <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
@@ -746,7 +774,10 @@
       <c r="I10" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="1"/>
+      <c r="J10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="1"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -754,9 +785,7 @@
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
-      <c r="D11" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D11" s="1"/>
       <c r="E11" s="1" t="n">
         <v>0</v>
       </c>
@@ -772,7 +801,10 @@
       <c r="I11" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="1"/>
+      <c r="J11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="1"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -797,21 +829,28 @@
         <v>0</v>
       </c>
       <c r="H12" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I12" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="J12" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="J12" s="1" t="s">
-        <v>12</v>
+      <c r="K12" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
         <v>45973</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+      <c r="B13" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="D13" s="1" t="n">
         <v>0</v>
       </c>
@@ -830,7 +869,12 @@
       <c r="I13" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J13" s="1"/>
+      <c r="J13" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -843,25 +887,28 @@
         <v>0</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H14" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>15</v>
+      <c r="K14" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="15">
@@ -870,9 +917,7 @@
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
-      <c r="D15" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D15" s="1"/>
       <c r="E15" s="1" t="n">
         <v>0</v>
       </c>
@@ -886,11 +931,12 @@
         <v>0</v>
       </c>
       <c r="I15" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="1"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -906,10 +952,10 @@
         <v>0</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>0</v>
@@ -918,10 +964,13 @@
         <v>0</v>
       </c>
       <c r="I16" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>11</v>
+        <v>1200</v>
+      </c>
+      <c r="J16" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="17">
@@ -932,10 +981,10 @@
         <v>0</v>
       </c>
       <c r="C17" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0</v>
@@ -950,10 +999,13 @@
         <v>0</v>
       </c>
       <c r="I17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="J17" s="1" t="s">
-        <v>16</v>
+      <c r="K17" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="18">
@@ -962,9 +1014,7 @@
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
-      <c r="D18" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D18" s="1"/>
       <c r="E18" s="1" t="n">
         <v>0</v>
       </c>
@@ -980,7 +1030,10 @@
       <c r="I18" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J18" s="1"/>
+      <c r="J18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="1"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -988,9 +1041,7 @@
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
-      <c r="D19" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D19" s="1"/>
       <c r="E19" s="1" t="n">
         <v>0</v>
       </c>
@@ -1006,7 +1057,10 @@
       <c r="I19" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J19" s="1"/>
+      <c r="J19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1016,13 +1070,13 @@
         <v>0</v>
       </c>
       <c r="C20" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="D20" s="1" t="n">
         <v>1200</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>0</v>
@@ -1034,10 +1088,13 @@
         <v>0</v>
       </c>
       <c r="I20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="1" t="n">
         <v>200</v>
       </c>
-      <c r="J20" s="1" t="s">
-        <v>17</v>
+      <c r="K20" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="21">
@@ -1046,9 +1103,7 @@
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
-      <c r="D21" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D21" s="1"/>
       <c r="E21" s="1" t="n">
         <v>0</v>
       </c>
@@ -1064,7 +1119,10 @@
       <c r="I21" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J21" s="1"/>
+      <c r="J21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="1"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1072,9 +1130,7 @@
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
-      <c r="D22" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D22" s="1"/>
       <c r="E22" s="1" t="n">
         <v>0</v>
       </c>
@@ -1090,7 +1146,10 @@
       <c r="I22" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J22" s="1"/>
+      <c r="J22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="1"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1098,9 +1157,7 @@
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
-      <c r="D23" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D23" s="1"/>
       <c r="E23" s="1" t="n">
         <v>0</v>
       </c>
@@ -1116,7 +1173,10 @@
       <c r="I23" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J23" s="1"/>
+      <c r="J23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="1"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1132,22 +1192,25 @@
         <v>0</v>
       </c>
       <c r="E24" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G24" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I24" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>11</v>
+        <v>1200</v>
+      </c>
+      <c r="J24" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="25">
@@ -1155,31 +1218,34 @@
         <v>45985</v>
       </c>
       <c r="B25" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C25" s="1" t="n">
         <v>1200</v>
       </c>
       <c r="D25" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E25" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G25" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H25" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="1" t="n">
         <v>300</v>
       </c>
-      <c r="J25" s="1" t="s">
-        <v>18</v>
+      <c r="K25" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="26">
@@ -1188,9 +1254,7 @@
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
-      <c r="D26" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D26" s="1"/>
       <c r="E26" s="1" t="n">
         <v>0</v>
       </c>
@@ -1206,7 +1270,10 @@
       <c r="I26" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J26" s="1"/>
+      <c r="J26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="1"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1214,9 +1281,7 @@
       </c>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
-      <c r="D27" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D27" s="1"/>
       <c r="E27" s="1" t="n">
         <v>0</v>
       </c>
@@ -1230,10 +1295,13 @@
         <v>0</v>
       </c>
       <c r="I27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="J27" s="1" t="s">
-        <v>11</v>
+      <c r="K27" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="28">
@@ -1242,9 +1310,7 @@
       </c>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
-      <c r="D28" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D28" s="1"/>
       <c r="E28" s="1" t="n">
         <v>0</v>
       </c>
@@ -1260,7 +1326,10 @@
       <c r="I28" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J28" s="1"/>
+      <c r="J28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="1"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1268,9 +1337,7 @@
       </c>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
-      <c r="D29" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="D29" s="1"/>
       <c r="E29" s="1" t="n">
         <v>0</v>
       </c>
@@ -1286,20 +1353,23 @@
       <c r="I29" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J29" s="1"/>
+      <c r="J29" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="1"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
         <v>45990</v>
       </c>
       <c r="B30" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C30" s="1" t="n">
         <v>1200</v>
       </c>
       <c r="D30" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>0</v>
@@ -1314,10 +1384,13 @@
         <v>0</v>
       </c>
       <c r="I30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="1" t="n">
         <v>200</v>
       </c>
-      <c r="J30" s="1" t="s">
-        <v>19</v>
+      <c r="K30" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="31">
@@ -1334,27 +1407,30 @@
         <v>0</v>
       </c>
       <c r="E31" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F31" s="1" t="n">
         <v>1200</v>
       </c>
       <c r="G31" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H31" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="J31" s="1" t="s">
-        <v>14</v>
+      <c r="K31" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B32" s="3" t="str">
         <f>SUM(B2:F31)</f>

</xml_diff>

<commit_message>
fix issue with room titles in reservation changes
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -56,31 +56,28 @@
     <t xml:space="preserve">Keydrops today: 1600</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: 513, 515</t>
+    <t xml:space="preserve">Keydrops today: 310</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 716, 513</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1615, 1600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1713</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1713, 716</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 814, 1713, 513</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 814, 1713</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 513</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 716</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 310</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1615, 1600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1713</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1713, 716</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814, 1713, 513</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814, 1713</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -619,7 +616,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H5" s="1" t="n">
         <v>1200</v>
@@ -628,10 +625,10 @@
         <v>0</v>
       </c>
       <c r="J5" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -692,9 +689,15 @@
       <c r="A8" s="2" t="n">
         <v>45968</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
+      <c r="B8" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="E8" s="1" t="n">
         <v>0</v>
       </c>
@@ -714,7 +717,7 @@
         <v>100</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -737,7 +740,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H9" s="1" t="n">
         <v>0</v>
@@ -746,10 +749,10 @@
         <v>0</v>
       </c>
       <c r="J9" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -873,7 +876,7 @@
         <v>100</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
@@ -905,10 +908,10 @@
         <v>0</v>
       </c>
       <c r="J14" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15">
@@ -970,7 +973,7 @@
         <v>200</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17">
@@ -1005,7 +1008,7 @@
         <v>100</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18">
@@ -1058,9 +1061,11 @@
         <v>0</v>
       </c>
       <c r="J19" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1094,7 +1099,7 @@
         <v>200</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">
@@ -1183,7 +1188,7 @@
         <v>45984</v>
       </c>
       <c r="B24" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="C24" s="1" t="n">
         <v>0</v>
@@ -1210,7 +1215,7 @@
         <v>200</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25">
@@ -1245,7 +1250,7 @@
         <v>300</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26">
@@ -1335,9 +1340,15 @@
       <c r="A29" s="2" t="n">
         <v>45989</v>
       </c>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
+      <c r="B29" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C29" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="E29" s="1" t="n">
         <v>0</v>
       </c>
@@ -1354,9 +1365,11 @@
         <v>0</v>
       </c>
       <c r="J29" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1390,7 +1403,7 @@
         <v>200</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31">
@@ -1425,12 +1438,12 @@
         <v>100</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B32" s="3" t="str">
         <f>SUM(B2:F31)</f>

</xml_diff>

<commit_message>
fix error caused by additional context parameter
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,12 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t xml:space="preserve">date</t>
   </si>
   <si>
-    <t xml:space="preserve">310</t>
+    <t xml:space="preserve">301</t>
   </si>
   <si>
     <t xml:space="preserve">814</t>
@@ -56,7 +56,10 @@
     <t xml:space="preserve">Keydrops today: 1600</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: 310</t>
+    <t xml:space="preserve">Keydrops today: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 301</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 716, 513</t>
@@ -69,6 +72,9 @@
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 1713, 716</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 301, 1615, 1600</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 814, 1713, 513</t>
@@ -635,9 +641,15 @@
       <c r="A6" s="2" t="n">
         <v>45966</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
+      <c r="B6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
@@ -656,7 +668,9 @@
       <c r="J6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="1"/>
+      <c r="K6" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -717,7 +731,7 @@
         <v>100</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -752,7 +766,7 @@
         <v>200</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -876,7 +890,7 @@
         <v>100</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
@@ -911,7 +925,7 @@
         <v>200</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
@@ -973,7 +987,7 @@
         <v>200</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17">
@@ -1008,16 +1022,22 @@
         <v>100</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
         <v>45978</v>
       </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
+      <c r="B18" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="E18" s="1" t="n">
         <v>0</v>
       </c>
@@ -1034,9 +1054,11 @@
         <v>0</v>
       </c>
       <c r="J18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1061,11 +1083,9 @@
         <v>0</v>
       </c>
       <c r="J19" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K19" s="1"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1099,7 +1119,7 @@
         <v>200</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21">
@@ -1212,10 +1232,10 @@
         <v>1200</v>
       </c>
       <c r="J24" s="1" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25">
@@ -1250,7 +1270,7 @@
         <v>300</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26">
@@ -1368,7 +1388,7 @@
         <v>100</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30">
@@ -1403,7 +1423,7 @@
         <v>200</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="31">
@@ -1438,12 +1458,12 @@
         <v>100</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B32" s="3" t="str">
         <f>SUM(B2:F31)</f>

</xml_diff>

<commit_message>
fix group id argument in 2pm line message
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 716, 513</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 301, 716, 513</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 1615, 1600</t>
@@ -898,7 +901,7 @@
         <v>45974</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="C14" s="1" t="n">
         <v>0</v>
@@ -922,10 +925,10 @@
         <v>0</v>
       </c>
       <c r="J14" s="1" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15">
@@ -987,7 +990,7 @@
         <v>200</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17">
@@ -1022,7 +1025,7 @@
         <v>100</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18">
@@ -1119,7 +1122,7 @@
         <v>200</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">
@@ -1235,7 +1238,7 @@
         <v>300</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25">
@@ -1270,7 +1273,7 @@
         <v>300</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26">
@@ -1423,7 +1426,7 @@
         <v>200</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="31">
@@ -1458,12 +1461,12 @@
         <v>100</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B32" s="3" t="str">
         <f>SUM(B2:F31)</f>

</xml_diff>

<commit_message>
fix another non-reservation email type
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -77,6 +77,9 @@
     <t xml:space="preserve">Keydrops today: 1713, 716</t>
   </si>
   <si>
+    <t xml:space="preserve">Keydrops today: 716</t>
+  </si>
+  <si>
     <t xml:space="preserve">Keydrops today: 301, 1615, 1600</t>
   </si>
   <si>
@@ -86,7 +89,7 @@
     <t xml:space="preserve">Keydrops today: 814, 1713</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: 513</t>
+    <t xml:space="preserve">Keydrops today: 1615, 513</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -1183,11 +1186,17 @@
       <c r="A23" s="2" t="n">
         <v>45983</v>
       </c>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
+      <c r="B23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="E23" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F23" s="1" t="n">
         <v>0</v>
@@ -1202,9 +1211,11 @@
         <v>0</v>
       </c>
       <c r="J23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1238,7 +1249,7 @@
         <v>300</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25">
@@ -1273,7 +1284,7 @@
         <v>300</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26">
@@ -1326,24 +1337,28 @@
         <v>0</v>
       </c>
       <c r="J27" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K27" s="1"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
         <v>45988</v>
       </c>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
+      <c r="B28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="E28" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G28" s="1" t="n">
         <v>0</v>
@@ -1355,9 +1370,11 @@
         <v>0</v>
       </c>
       <c r="J28" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1426,7 +1443,7 @@
         <v>200</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31">
@@ -1458,15 +1475,15 @@
         <v>0</v>
       </c>
       <c r="J31" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B32" s="3" t="str">
         <f>SUM(B2:F31)</f>

</xml_diff>

<commit_message>
replies and manual additions
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,9 +12,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t xml:space="preserve">date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renai Casa 2F-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Casa 2-3</t>
   </si>
   <si>
     <t xml:space="preserve">301</t>
@@ -502,6 +508,12 @@
       <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -526,16 +538,22 @@
         <v>0</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="J2" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="K2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>11</v>
+      <c r="M2" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -555,22 +573,28 @@
         <v>0</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H3" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I3" s="1" t="n">
         <v>0</v>
       </c>
       <c r="J3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>12</v>
+      <c r="M3" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -599,13 +623,19 @@
         <v>0</v>
       </c>
       <c r="I4" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="L4" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>13</v>
+      <c r="M4" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -619,28 +649,34 @@
         <v>0</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="J5" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="K5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="K5" s="1" t="s">
-        <v>11</v>
+      <c r="M5" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -674,8 +710,14 @@
       <c r="J6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>14</v>
+      <c r="K6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -685,12 +727,8 @@
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
-      <c r="E7" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
       <c r="G7" s="1" t="n">
         <v>0</v>
       </c>
@@ -703,20 +741,26 @@
       <c r="J7" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K7" s="1"/>
+      <c r="K7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="1"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C8" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>0</v>
@@ -734,10 +778,16 @@
         <v>0</v>
       </c>
       <c r="J8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="K8" s="1" t="s">
-        <v>15</v>
+      <c r="M8" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -754,7 +804,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>0</v>
@@ -766,13 +816,19 @@
         <v>0</v>
       </c>
       <c r="I9" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="1" t="n">
         <v>200</v>
       </c>
-      <c r="K9" s="1" t="s">
-        <v>16</v>
+      <c r="M9" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -782,12 +838,8 @@
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
-      <c r="E10" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
       <c r="G10" s="1" t="n">
         <v>0</v>
       </c>
@@ -800,7 +852,13 @@
       <c r="J10" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="1"/>
+      <c r="K10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="1"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -809,12 +867,8 @@
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
       <c r="G11" s="1" t="n">
         <v>0</v>
       </c>
@@ -827,7 +881,13 @@
       <c r="J11" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="1"/>
+      <c r="K11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="1"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -855,13 +915,19 @@
         <v>0</v>
       </c>
       <c r="I12" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="L12" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="K12" s="1" t="s">
-        <v>13</v>
+      <c r="M12" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -869,13 +935,13 @@
         <v>45973</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>0</v>
@@ -893,10 +959,16 @@
         <v>0</v>
       </c>
       <c r="J13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="K13" s="1" t="s">
-        <v>15</v>
+      <c r="M13" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="14">
@@ -904,16 +976,16 @@
         <v>45974</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C14" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F14" s="1" t="n">
         <v>0</v>
@@ -925,13 +997,19 @@
         <v>0</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="1" t="n">
         <v>300</v>
       </c>
-      <c r="K14" s="1" t="s">
-        <v>17</v>
+      <c r="M14" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="15">
@@ -941,12 +1019,8 @@
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
-      <c r="E15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
       <c r="G15" s="1" t="n">
         <v>0</v>
       </c>
@@ -959,7 +1033,13 @@
       <c r="J15" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="1"/>
+      <c r="K15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="1"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -978,22 +1058,28 @@
         <v>0</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H16" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I16" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="L16" s="1" t="n">
         <v>200</v>
       </c>
-      <c r="K16" s="1" t="s">
-        <v>18</v>
+      <c r="M16" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="17">
@@ -1007,13 +1093,13 @@
         <v>0</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>0</v>
@@ -1025,10 +1111,16 @@
         <v>0</v>
       </c>
       <c r="J17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="K17" s="1" t="s">
-        <v>19</v>
+      <c r="M17" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="18">
@@ -1036,13 +1128,13 @@
         <v>45978</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>0</v>
@@ -1060,10 +1152,16 @@
         <v>0</v>
       </c>
       <c r="J18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="K18" s="1" t="s">
-        <v>15</v>
+      <c r="M18" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="19">
@@ -1073,12 +1171,8 @@
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
-      <c r="E19" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
       <c r="G19" s="1" t="n">
         <v>0</v>
       </c>
@@ -1091,7 +1185,13 @@
       <c r="J19" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="1"/>
+      <c r="K19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="1"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1104,16 +1204,16 @@
         <v>0</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G20" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H20" s="1" t="n">
         <v>0</v>
@@ -1122,10 +1222,16 @@
         <v>0</v>
       </c>
       <c r="J20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="1" t="n">
         <v>200</v>
       </c>
-      <c r="K20" s="1" t="s">
-        <v>20</v>
+      <c r="M20" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="21">
@@ -1135,12 +1241,8 @@
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
-      <c r="E21" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
       <c r="G21" s="1" t="n">
         <v>0</v>
       </c>
@@ -1153,7 +1255,13 @@
       <c r="J21" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K21" s="1"/>
+      <c r="K21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="1"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1162,12 +1270,8 @@
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
-      <c r="E22" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
       <c r="G22" s="1" t="n">
         <v>0</v>
       </c>
@@ -1180,7 +1284,13 @@
       <c r="J22" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="1"/>
+      <c r="K22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="1"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1196,13 +1306,13 @@
         <v>0</v>
       </c>
       <c r="E23" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F23" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H23" s="1" t="n">
         <v>0</v>
@@ -1211,10 +1321,16 @@
         <v>0</v>
       </c>
       <c r="J23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="K23" s="1" t="s">
-        <v>21</v>
+      <c r="M23" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="24">
@@ -1222,34 +1338,40 @@
         <v>45984</v>
       </c>
       <c r="B24" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C24" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E24" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G24" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I24" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J24" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="L24" s="1" t="n">
         <v>300</v>
       </c>
-      <c r="K24" s="1" t="s">
-        <v>22</v>
+      <c r="M24" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="25">
@@ -1260,31 +1382,37 @@
         <v>0</v>
       </c>
       <c r="C25" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="D25" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E25" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G25" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H25" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I25" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="1" t="n">
         <v>300</v>
       </c>
-      <c r="K25" s="1" t="s">
-        <v>23</v>
+      <c r="M25" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="26">
@@ -1294,12 +1422,8 @@
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
-      <c r="E26" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
       <c r="G26" s="1" t="n">
         <v>0</v>
       </c>
@@ -1312,7 +1436,13 @@
       <c r="J26" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K26" s="1"/>
+      <c r="K26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="1"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1321,12 +1451,8 @@
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
-      <c r="E27" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
       <c r="G27" s="1" t="n">
         <v>0</v>
       </c>
@@ -1339,7 +1465,13 @@
       <c r="J27" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="K27" s="1"/>
+      <c r="K27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="1"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1358,22 +1490,28 @@
         <v>0</v>
       </c>
       <c r="F28" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G28" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H28" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I28" s="1" t="n">
         <v>0</v>
       </c>
       <c r="J28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="K28" s="1" t="s">
-        <v>12</v>
+      <c r="M28" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="29">
@@ -1381,13 +1519,13 @@
         <v>45989</v>
       </c>
       <c r="B29" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C29" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E29" s="1" t="n">
         <v>0</v>
@@ -1405,10 +1543,16 @@
         <v>0</v>
       </c>
       <c r="J29" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="K29" s="1" t="s">
-        <v>15</v>
+      <c r="M29" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="30">
@@ -1419,16 +1563,16 @@
         <v>0</v>
       </c>
       <c r="C30" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="D30" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E30" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F30" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G30" s="1" t="n">
         <v>0</v>
@@ -1440,10 +1584,16 @@
         <v>0</v>
       </c>
       <c r="J30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="1" t="n">
         <v>200</v>
       </c>
-      <c r="K30" s="1" t="s">
-        <v>24</v>
+      <c r="M30" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="31">
@@ -1463,27 +1613,33 @@
         <v>0</v>
       </c>
       <c r="F31" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G31" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H31" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I31" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="1" t="n">
         <v>200</v>
       </c>
-      <c r="K31" s="1" t="s">
-        <v>25</v>
+      <c r="M31" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B32" s="3" t="str">
         <f>SUM(B2:F31)</f>

</xml_diff>

<commit_message>
fix line message december dates
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -53,49 +53,52 @@
     <t xml:space="preserve">keycard_drop_rooms</t>
   </si>
   <si>
+    <t xml:space="preserve">Keydrops today: Casa 2-3, 716</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: Renai Casa 2F-2, 1713, 515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1615</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 814, 716, 1600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 301, 515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 513</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: Casa 2-3, 814</t>
+  </si>
+  <si>
     <t xml:space="preserve">Keydrops today: 515</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: 1615</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: </t>
+    <t xml:space="preserve">Keydrops today: 1713</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 716, 513</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 814, 1600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 814, 1713</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1615, 1600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 716</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 301</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: 716, 513</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 301, 716, 513</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1615, 1600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1713</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1713, 716</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 716</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 301, 1615, 1600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814, 1713, 513</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814, 1713</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1615, 513</t>
+    <t xml:space="preserve">Keydrops today: 814, 1713, 1615, 515, 1600</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -517,13 +520,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>0</v>
@@ -535,7 +538,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H2" s="1" t="n">
         <v>0</v>
@@ -544,13 +547,13 @@
         <v>0</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="K2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>13</v>
@@ -558,28 +561,18 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45963</v>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>45993</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
       <c r="G3" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H3" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I3" s="1" t="n">
         <v>0</v>
@@ -591,18 +584,16 @@
         <v>0</v>
       </c>
       <c r="L3" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M3" s="1"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45964</v>
+        <v>45994</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>0</v>
@@ -614,7 +605,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>0</v>
@@ -626,37 +617,27 @@
         <v>0</v>
       </c>
       <c r="J4" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="K4" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="L4" s="1" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45965</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="1" t="n">
-        <v>1200</v>
-      </c>
+        <v>45995</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
       <c r="G5" s="1" t="n">
         <v>0</v>
       </c>
@@ -667,21 +648,19 @@
         <v>0</v>
       </c>
       <c r="J5" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="K5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L5" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>13</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M5" s="1"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45966</v>
+        <v>45996</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0</v>
@@ -702,7 +681,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I6" s="1" t="n">
         <v>0</v>
@@ -714,23 +693,33 @@
         <v>0</v>
       </c>
       <c r="L6" s="1" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45967</v>
-      </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
+        <v>45997</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G7" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H7" s="1" t="n">
         <v>0</v>
@@ -742,16 +731,18 @@
         <v>0</v>
       </c>
       <c r="K7" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="L7" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="1"/>
+        <v>300</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45968</v>
+        <v>45998</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0</v>
@@ -778,13 +769,13 @@
         <v>0</v>
       </c>
       <c r="J8" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="K8" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="M8" s="1" t="s">
         <v>17</v>
@@ -792,7 +783,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45969</v>
+        <v>45999</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0</v>
@@ -810,7 +801,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H9" s="1" t="n">
         <v>0</v>
@@ -825,7 +816,7 @@
         <v>0</v>
       </c>
       <c r="L9" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="M9" s="1" t="s">
         <v>18</v>
@@ -833,13 +824,23 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45970</v>
-      </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
+        <v>46000</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G10" s="1" t="n">
         <v>0</v>
       </c>
@@ -856,13 +857,15 @@
         <v>0</v>
       </c>
       <c r="L10" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="1"/>
+        <v>200</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45971</v>
+        <v>46001</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -885,29 +888,21 @@
         <v>0</v>
       </c>
       <c r="L11" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>45972</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46002</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
       <c r="G12" s="1" t="n">
         <v>0</v>
       </c>
@@ -921,34 +916,22 @@
         <v>0</v>
       </c>
       <c r="K12" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="L12" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M12" s="1" t="s">
-        <v>15</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M12" s="1"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>45973</v>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="1" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46003</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
       <c r="G13" s="1" t="n">
         <v>0</v>
       </c>
@@ -965,15 +948,13 @@
         <v>0</v>
       </c>
       <c r="L13" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M13" s="1" t="s">
-        <v>17</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M13" s="1"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>45974</v>
+        <v>46004</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0</v>
@@ -982,22 +963,22 @@
         <v>0</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H14" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J14" s="1" t="n">
         <v>0</v>
@@ -1006,44 +987,56 @@
         <v>0</v>
       </c>
       <c r="L14" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>45975</v>
-      </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
+        <v>46005</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G15" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I15" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J15" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="K15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="1"/>
+        <v>200</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>45976</v>
+        <v>46006</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0</v>
@@ -1055,7 +1048,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F16" s="1" t="n">
         <v>0</v>
@@ -1064,7 +1057,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I16" s="1" t="n">
         <v>0</v>
@@ -1079,28 +1072,18 @@
         <v>200</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>45977</v>
-      </c>
-      <c r="B17" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="1" t="n">
-        <v>1200</v>
-      </c>
+        <v>46007</v>
+      </c>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
       <c r="G17" s="1" t="n">
         <v>0</v>
       </c>
@@ -1117,31 +1100,19 @@
         <v>0</v>
       </c>
       <c r="L17" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M17" s="1" t="s">
-        <v>21</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M17" s="1"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>45978</v>
-      </c>
-      <c r="B18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="1" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46008</v>
+      </c>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
       <c r="G18" s="1" t="n">
         <v>0</v>
       </c>
@@ -1161,18 +1132,28 @@
         <v>100</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>45979</v>
-      </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
+        <v>46009</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G19" s="1" t="n">
         <v>0</v>
       </c>
@@ -1189,13 +1170,15 @@
         <v>0</v>
       </c>
       <c r="L19" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="1"/>
+        <v>200</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>45980</v>
+        <v>46010</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0</v>
@@ -1210,13 +1193,13 @@
         <v>0</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G20" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H20" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I20" s="1" t="n">
         <v>0</v>
@@ -1225,18 +1208,18 @@
         <v>0</v>
       </c>
       <c r="K20" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="L20" s="1" t="n">
         <v>200</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>45981</v>
+        <v>46011</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1265,13 +1248,23 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>45982</v>
-      </c>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
+        <v>46012</v>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F22" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G22" s="1" t="n">
         <v>0</v>
       </c>
@@ -1288,13 +1281,15 @@
         <v>0</v>
       </c>
       <c r="L22" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" s="1"/>
+        <v>200</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>45983</v>
+        <v>46013</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>0</v>
@@ -1309,16 +1304,16 @@
         <v>0</v>
       </c>
       <c r="F23" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G23" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H23" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J23" s="1" t="n">
         <v>0</v>
@@ -1327,15 +1322,13 @@
         <v>0</v>
       </c>
       <c r="L23" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>23</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M23" s="1"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>45984</v>
+        <v>46014</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>0</v>
@@ -1344,7 +1337,7 @@
         <v>0</v>
       </c>
       <c r="D24" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E24" s="1" t="n">
         <v>0</v>
@@ -1356,27 +1349,27 @@
         <v>0</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I24" s="1" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="K24" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="L24" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>45985</v>
+        <v>46015</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>0</v>
@@ -1388,19 +1381,19 @@
         <v>0</v>
       </c>
       <c r="E25" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G25" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H25" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I25" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J25" s="1" t="n">
         <v>0</v>
@@ -1409,23 +1402,33 @@
         <v>0</v>
       </c>
       <c r="L25" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>45986</v>
-      </c>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
+        <v>46016</v>
+      </c>
+      <c r="B26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G26" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H26" s="1" t="n">
         <v>0</v>
@@ -1440,19 +1443,31 @@
         <v>0</v>
       </c>
       <c r="L26" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M26" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>45987</v>
-      </c>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
+        <v>46017</v>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G27" s="1" t="n">
         <v>0</v>
       </c>
@@ -1469,34 +1484,26 @@
         <v>0</v>
       </c>
       <c r="L27" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M27" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>45988</v>
-      </c>
-      <c r="B28" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46018</v>
+      </c>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
       <c r="G28" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H28" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I28" s="1" t="n">
         <v>0</v>
@@ -1508,15 +1515,13 @@
         <v>0</v>
       </c>
       <c r="L28" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M28" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M28" s="1"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>45989</v>
+        <v>46019</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>0</v>
@@ -1525,39 +1530,39 @@
         <v>0</v>
       </c>
       <c r="D29" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E29" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F29" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G29" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H29" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I29" s="1" t="n">
         <v>0</v>
       </c>
       <c r="J29" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="K29" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="L29" s="1" t="n">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>45990</v>
+        <v>46020</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>0</v>
@@ -1569,10 +1574,10 @@
         <v>0</v>
       </c>
       <c r="E30" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F30" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G30" s="1" t="n">
         <v>0</v>
@@ -1581,7 +1586,7 @@
         <v>0</v>
       </c>
       <c r="I30" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J30" s="1" t="n">
         <v>0</v>
@@ -1590,39 +1595,29 @@
         <v>0</v>
       </c>
       <c r="L30" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>45991</v>
-      </c>
-      <c r="B31" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46021</v>
+      </c>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
       <c r="G31" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H31" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I31" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J31" s="1" t="n">
         <v>0</v>
@@ -1631,35 +1626,62 @@
         <v>0</v>
       </c>
       <c r="L31" s="1" t="n">
-        <v>200</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>27</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M31" s="1"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B32" s="3" t="str">
-        <f>SUM(B2:F31)</f>
-      </c>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3" t="str">
-        <f>SUM(G2:H31)</f>
-      </c>
-      <c r="H32" s="3"/>
-      <c r="I32" s="3" t="str">
-        <f>SUM(I2:I31)</f>
+      <c r="A32" s="2" t="n">
+        <v>46022</v>
+      </c>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="1"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" s="3" t="str">
+        <f>SUM(B2:F32)</f>
+      </c>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3" t="str">
+        <f>SUM(G2:H32)</f>
+      </c>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3" t="str">
+        <f>SUM(I2:I32)</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="G33:H33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
manually add a guest
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: Renai Casa 2F-2</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 1713</t>
@@ -898,11 +901,21 @@
       <c r="A12" s="2" t="n">
         <v>46002</v>
       </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
+      <c r="B12" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G12" s="1" t="n">
         <v>0</v>
       </c>
@@ -919,9 +932,11 @@
         <v>0</v>
       </c>
       <c r="L12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -990,7 +1005,7 @@
         <v>100</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15">
@@ -1031,7 +1046,7 @@
         <v>200</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16">
@@ -1072,7 +1087,7 @@
         <v>200</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17">
@@ -1173,7 +1188,7 @@
         <v>200</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20">
@@ -1214,7 +1229,7 @@
         <v>200</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21">
@@ -1446,7 +1461,7 @@
         <v>100</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27">
@@ -1487,7 +1502,7 @@
         <v>100</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="28">
@@ -1557,7 +1572,7 @@
         <v>500</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30">
@@ -1661,7 +1676,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B33" s="3" t="str">
         <f>SUM(B2:F32)</f>

</xml_diff>

<commit_message>
combine funtions in utils + delint
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -101,7 +101,7 @@
     <t xml:space="preserve">Keydrops today: Renai Casa 2F-2, 515</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: 716</t>
+    <t xml:space="preserve">Keydrops today: 716, 513</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 301</t>
@@ -1455,7 +1455,7 @@
         <v>0</v>
       </c>
       <c r="I26" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J26" s="1" t="n">
         <v>0</v>
@@ -1464,7 +1464,7 @@
         <v>0</v>
       </c>
       <c r="L26" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="M26" s="1" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
fix issue with multiple change requests to same reservation
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -53,58 +53,37 @@
     <t xml:space="preserve">keycard_drop_rooms</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: Casa 2-3, 716</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: Renai Casa 2F-2, 1713, 515</t>
+    <t xml:space="preserve">Keydrops today: 515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 301, 716, 513</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 1615</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: 814, 716, 1600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 301, 515</t>
+    <t xml:space="preserve">Keydrops today: 1615, 513</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 814, 1713</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 301</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1713</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 513</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: Casa 2-3, 814</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 515</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: Renai Casa 2F-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1713</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: Renai Casa 2F-2, 716, 513</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 301, 814, 1600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814, 513, 515</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1713, 1615, 1600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: Renai Casa 2F-2, 1713, 513</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 716, 513</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 301</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814, 1713, 1615, 515, 1600</t>
+    <t xml:space="preserve">Keydrops today: 1713, 1615</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 814</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: Renai Casa 2F-2, 1600</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -526,13 +505,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>0</v>
@@ -544,7 +523,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H2" s="1" t="n">
         <v>0</v>
@@ -553,13 +532,13 @@
         <v>0</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="K2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>13</v>
@@ -567,21 +546,31 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45993</v>
-      </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
+        <v>46024</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>1200</v>
+      </c>
       <c r="G3" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H3" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J3" s="1" t="n">
         <v>0</v>
@@ -590,16 +579,18 @@
         <v>0</v>
       </c>
       <c r="L3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="1"/>
+        <v>300</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45994</v>
+        <v>46025</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>0</v>
@@ -611,39 +602,49 @@
         <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H4" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="J4" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="K4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L4" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45995</v>
-      </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
+        <v>46026</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G5" s="1" t="n">
         <v>0</v>
       </c>
@@ -654,40 +655,32 @@
         <v>0</v>
       </c>
       <c r="J5" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="K5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45996</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46027</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
       <c r="G6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I6" s="1" t="n">
         <v>0</v>
@@ -699,15 +692,13 @@
         <v>0</v>
       </c>
       <c r="L6" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>15</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M6" s="1"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45997</v>
+        <v>46028</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0</v>
@@ -719,28 +710,28 @@
         <v>0</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H7" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I7" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J7" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K7" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="L7" s="1" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="M7" s="1" t="s">
         <v>16</v>
@@ -748,7 +739,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45998</v>
+        <v>46029</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0</v>
@@ -757,13 +748,13 @@
         <v>0</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>0</v>
@@ -775,7 +766,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="K8" s="1" t="n">
         <v>0</v>
@@ -789,7 +780,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45999</v>
+        <v>46030</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0</v>
@@ -798,7 +789,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>0</v>
@@ -813,7 +804,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J9" s="1" t="n">
         <v>0</v>
@@ -830,19 +821,19 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46000</v>
+        <v>46031</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>0</v>
@@ -860,29 +851,37 @@
         <v>0</v>
       </c>
       <c r="K10" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="L10" s="1" t="n">
-        <v>200</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>19</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M10" s="1"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46001</v>
-      </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
+        <v>46032</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G11" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I11" s="1" t="n">
         <v>0</v>
@@ -897,15 +896,15 @@
         <v>100</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46002</v>
+        <v>46033</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C12" s="1" t="n">
         <v>0</v>
@@ -929,7 +928,7 @@
         <v>0</v>
       </c>
       <c r="J12" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="K12" s="1" t="n">
         <v>0</v>
@@ -938,12 +937,12 @@
         <v>100</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46003</v>
+        <v>46034</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -966,13 +965,15 @@
         <v>0</v>
       </c>
       <c r="L13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46004</v>
+        <v>46035</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0</v>
@@ -1008,15 +1009,15 @@
         <v>100</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46005</v>
+        <v>46036</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C15" s="1" t="n">
         <v>0</v>
@@ -1031,7 +1032,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H15" s="1" t="n">
         <v>0</v>
@@ -1040,37 +1041,27 @@
         <v>1200</v>
       </c>
       <c r="J15" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="K15" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46006</v>
-      </c>
-      <c r="B16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="1" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E16" s="1" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F16" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46037</v>
+      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
       <c r="G16" s="1" t="n">
         <v>0</v>
       </c>
@@ -1084,29 +1075,37 @@
         <v>0</v>
       </c>
       <c r="K16" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="L16" s="1" t="n">
-        <v>300</v>
-      </c>
-      <c r="M16" s="1" t="s">
-        <v>24</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M16" s="1"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46007</v>
-      </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
+        <v>46038</v>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G17" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H17" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I17" s="1" t="n">
         <v>0</v>
@@ -1118,19 +1117,31 @@
         <v>0</v>
       </c>
       <c r="L17" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="1"/>
+        <v>200</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46008</v>
-      </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
+        <v>46039</v>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F18" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G18" s="1" t="n">
         <v>0</v>
       </c>
@@ -1147,16 +1158,18 @@
         <v>0</v>
       </c>
       <c r="L18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46009</v>
+        <v>46040</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>0</v>
@@ -1165,7 +1178,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F19" s="1" t="n">
         <v>0</v>
@@ -1177,45 +1190,35 @@
         <v>0</v>
       </c>
       <c r="I19" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J19" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="K19" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="L19" s="1" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46010</v>
-      </c>
-      <c r="B20" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="1" t="n">
-        <v>1200</v>
-      </c>
+        <v>46041</v>
+      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
       <c r="G20" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H20" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I20" s="1" t="n">
         <v>0</v>
@@ -1224,18 +1227,16 @@
         <v>0</v>
       </c>
       <c r="K20" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="L20" s="1" t="n">
-        <v>300</v>
-      </c>
-      <c r="M20" s="1" t="s">
-        <v>26</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M20" s="1"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46011</v>
+        <v>46042</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1264,19 +1265,19 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46012</v>
+        <v>46043</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C22" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="D22" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F22" s="1" t="n">
         <v>0</v>
@@ -1288,7 +1289,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J22" s="1" t="n">
         <v>0</v>
@@ -1297,31 +1298,21 @@
         <v>0</v>
       </c>
       <c r="L22" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46013</v>
-      </c>
-      <c r="B23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="1" t="n">
-        <v>1200</v>
-      </c>
+        <v>46044</v>
+      </c>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
       <c r="G23" s="1" t="n">
         <v>0</v>
       </c>
@@ -1329,7 +1320,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J23" s="1" t="n">
         <v>0</v>
@@ -1338,15 +1329,15 @@
         <v>0</v>
       </c>
       <c r="L23" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46014</v>
+        <v>46045</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>0</v>
@@ -1367,13 +1358,13 @@
         <v>0</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I24" s="1" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="K24" s="1" t="n">
         <v>0</v>
@@ -1382,33 +1373,23 @@
         <v>100</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46015</v>
-      </c>
-      <c r="B25" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46046</v>
+      </c>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
       <c r="G25" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H25" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I25" s="1" t="n">
         <v>0</v>
@@ -1420,39 +1401,27 @@
         <v>0</v>
       </c>
       <c r="L25" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>15</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M25" s="1"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46016</v>
-      </c>
-      <c r="B26" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46047</v>
+      </c>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
       <c r="G26" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H26" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I26" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J26" s="1" t="n">
         <v>0</v>
@@ -1461,31 +1430,21 @@
         <v>0</v>
       </c>
       <c r="L26" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46017</v>
-      </c>
-      <c r="B27" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="1" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E27" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46048</v>
+      </c>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
       <c r="G27" s="1" t="n">
         <v>0</v>
       </c>
@@ -1502,21 +1461,29 @@
         <v>0</v>
       </c>
       <c r="L27" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M27" s="1" t="s">
-        <v>29</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M27" s="1"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46018</v>
-      </c>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
+        <v>46049</v>
+      </c>
+      <c r="B28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="1" t="n">
+        <v>1200</v>
+      </c>
       <c r="G28" s="1" t="n">
         <v>0</v>
       </c>
@@ -1524,7 +1491,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J28" s="1" t="n">
         <v>0</v>
@@ -1533,13 +1500,15 @@
         <v>0</v>
       </c>
       <c r="L28" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M28" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46019</v>
+        <v>46050</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>0</v>
@@ -1554,7 +1523,7 @@
         <v>1200</v>
       </c>
       <c r="F29" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="G29" s="1" t="n">
         <v>0</v>
@@ -1566,37 +1535,27 @@
         <v>0</v>
       </c>
       <c r="J29" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="K29" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="L29" s="1" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46020</v>
-      </c>
-      <c r="B30" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46051</v>
+      </c>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
       <c r="G30" s="1" t="n">
         <v>0</v>
       </c>
@@ -1604,7 +1563,7 @@
         <v>0</v>
       </c>
       <c r="I30" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J30" s="1" t="n">
         <v>0</v>
@@ -1613,15 +1572,13 @@
         <v>0</v>
       </c>
       <c r="L30" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M30" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M30" s="1"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46021</v>
+        <v>46052</v>
       </c>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1650,7 +1607,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46022</v>
+        <v>46053</v>
       </c>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -1679,7 +1636,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B33" s="3" t="str">
         <f>SUM(B2:F32)</f>

</xml_diff>

<commit_message>
move files to folder and overwrite
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -53,40 +53,34 @@
     <t xml:space="preserve">keycard_drop_rooms</t>
   </si>
   <si>
+    <t xml:space="preserve">Keydrops today: 814, 1713</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 716</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1615</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: Renai Casa 2F-2, 814, 513, 515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 513</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1713, 716, 1615</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 814, 515</t>
+  </si>
+  <si>
     <t xml:space="preserve">Keydrops today: Casa 2-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: Renai Casa 2F-2, 1615</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 716</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1615, 1600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 515</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: Renai Casa 2F-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 1615</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814, 1615</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 814, 513, 515</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: 513</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keydrops today: Renai Casa 2F-2, 301, 716, 513</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -508,13 +502,13 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>0</v>
@@ -523,7 +517,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>0</v>
@@ -541,7 +535,7 @@
         <v>0</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>13</v>
@@ -549,10 +543,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46055</v>
+        <v>46083</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>0</v>
@@ -570,7 +564,7 @@
         <v>0</v>
       </c>
       <c r="H3" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I3" s="1" t="n">
         <v>0</v>
@@ -579,10 +573,10 @@
         <v>0</v>
       </c>
       <c r="K3" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="L3" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="M3" s="1" t="s">
         <v>14</v>
@@ -590,7 +584,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46056</v>
+        <v>46084</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>0</v>
@@ -602,7 +596,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>0</v>
@@ -617,7 +611,7 @@
         <v>0</v>
       </c>
       <c r="J4" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="K4" s="1" t="n">
         <v>0</v>
@@ -631,15 +625,25 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46057</v>
-      </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
+        <v>46085</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G5" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H5" s="1" t="n">
         <v>0</v>
@@ -654,13 +658,15 @@
         <v>0</v>
       </c>
       <c r="L5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46058</v>
+        <v>46086</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -683,13 +689,15 @@
         <v>0</v>
       </c>
       <c r="L6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46059</v>
+        <v>46087</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0</v>
@@ -701,13 +709,13 @@
         <v>0</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H7" s="1" t="n">
         <v>0</v>
@@ -722,15 +730,13 @@
         <v>0</v>
       </c>
       <c r="L7" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>16</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M7" s="1"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46060</v>
+        <v>46088</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0</v>
@@ -760,10 +766,10 @@
         <v>0</v>
       </c>
       <c r="K8" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="L8" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="M8" s="1" t="s">
         <v>17</v>
@@ -771,23 +777,13 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46061</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46089</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
       <c r="G9" s="1" t="n">
         <v>0</v>
       </c>
@@ -798,27 +794,35 @@
         <v>0</v>
       </c>
       <c r="J9" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="K9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>18</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M9" s="1"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46062</v>
-      </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
+        <v>46090</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G10" s="1" t="n">
         <v>0</v>
       </c>
@@ -826,30 +830,42 @@
         <v>0</v>
       </c>
       <c r="I10" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J10" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="K10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="1"/>
+        <v>400</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46063</v>
-      </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
+        <v>46091</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G11" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H11" s="1" t="n">
         <v>0</v>
@@ -861,32 +877,24 @@
         <v>0</v>
       </c>
       <c r="K11" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="L11" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46064</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="1" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F12" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46092</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
       <c r="G12" s="1" t="n">
         <v>0</v>
       </c>
@@ -894,7 +902,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J12" s="1" t="n">
         <v>0</v>
@@ -903,15 +911,13 @@
         <v>0</v>
       </c>
       <c r="L12" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M12" s="1" t="s">
-        <v>15</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M12" s="1"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46065</v>
+        <v>46093</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -934,13 +940,15 @@
         <v>0</v>
       </c>
       <c r="L13" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46066</v>
+        <v>46094</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -963,31 +971,19 @@
         <v>0</v>
       </c>
       <c r="L14" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M14" s="1" t="s">
-        <v>16</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M14" s="1"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46067</v>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>1200</v>
-      </c>
-      <c r="C15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46095</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
       <c r="G15" s="1" t="n">
         <v>0</v>
       </c>
@@ -1004,15 +1000,13 @@
         <v>0</v>
       </c>
       <c r="L15" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M15" s="1" t="s">
-        <v>19</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M15" s="1"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46068</v>
+        <v>46096</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0</v>
@@ -1033,7 +1027,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I16" s="1" t="n">
         <v>0</v>
@@ -1042,18 +1036,18 @@
         <v>0</v>
       </c>
       <c r="K16" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="L16" s="1" t="n">
         <v>100</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46069</v>
+        <v>46097</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1082,21 +1076,31 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46070</v>
-      </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
+        <v>46098</v>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G18" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H18" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I18" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J18" s="1" t="n">
         <v>0</v>
@@ -1105,21 +1109,33 @@
         <v>0</v>
       </c>
       <c r="L18" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46071</v>
-      </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
+        <v>46099</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G19" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H19" s="1" t="n">
         <v>0</v>
@@ -1134,13 +1150,15 @@
         <v>0</v>
       </c>
       <c r="L19" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46072</v>
+        <v>46100</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0</v>
@@ -1152,52 +1170,42 @@
         <v>0</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G20" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H20" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I20" s="1" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="K20" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46073</v>
-      </c>
-      <c r="B21" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="1" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E21" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46101</v>
+      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
       <c r="G21" s="1" t="n">
         <v>0</v>
       </c>
@@ -1220,7 +1228,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46074</v>
+        <v>46102</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>0</v>
@@ -1232,7 +1240,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="F22" s="1" t="n">
         <v>0</v>
@@ -1244,35 +1252,45 @@
         <v>0</v>
       </c>
       <c r="I22" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J22" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="K22" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="L22" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
+        <v>46103</v>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="1" t="n">
+        <v>1200</v>
+      </c>
       <c r="G23" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="H23" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I23" s="1" t="n">
         <v>0</v>
@@ -1284,13 +1302,15 @@
         <v>0</v>
       </c>
       <c r="L23" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="1"/>
+        <v>300</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46076</v>
+        <v>46104</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>0</v>
@@ -1311,27 +1331,27 @@
         <v>0</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I24" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J24" s="1" t="n">
         <v>0</v>
       </c>
       <c r="K24" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="L24" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46077</v>
+        <v>46105</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>0</v>
@@ -1343,7 +1363,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F25" s="1" t="n">
         <v>0</v>
@@ -1355,24 +1375,24 @@
         <v>0</v>
       </c>
       <c r="I25" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J25" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="K25" s="1" t="n">
         <v>0</v>
       </c>
       <c r="L25" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46078</v>
+        <v>46106</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1395,13 +1415,15 @@
         <v>0</v>
       </c>
       <c r="L26" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M26" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46079</v>
+        <v>46107</v>
       </c>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1424,13 +1446,15 @@
         <v>0</v>
       </c>
       <c r="L27" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M27" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46080</v>
+        <v>46108</v>
       </c>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1459,31 +1483,21 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46081</v>
-      </c>
-      <c r="B29" s="1" t="n">
-        <v>1200</v>
-      </c>
-      <c r="C29" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" s="1" t="n">
-        <v>0</v>
-      </c>
+        <v>46109</v>
+      </c>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
       <c r="G29" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="H29" s="1" t="n">
         <v>0</v>
       </c>
       <c r="I29" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="J29" s="1" t="n">
         <v>0</v>
@@ -1492,35 +1506,134 @@
         <v>0</v>
       </c>
       <c r="L29" s="1" t="n">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B30" s="3" t="str">
-        <f>SUM(B2:F29)</f>
-      </c>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-      <c r="G30" s="3" t="str">
-        <f>SUM(G2:H29)</f>
-      </c>
-      <c r="H30" s="3"/>
-      <c r="I30" s="3" t="str">
-        <f>SUM(I2:I29)</f>
+      <c r="A30" s="2" t="n">
+        <v>46110</v>
+      </c>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="1"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46111</v>
+      </c>
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="1"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="1" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B33" s="3" t="str">
+        <f>SUM(B2:F32)</f>
+      </c>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3" t="str">
+        <f>SUM(G2:H32)</f>
+      </c>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3" t="str">
+        <f>SUM(I2:I32)</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="G33:H33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
add a reminders check at t the end to catch cancelations and changes that didn't have any emails
</commit_message>
<xml_diff>
--- a/data/this_months_payment_schedule.xlsx
+++ b/data/this_months_payment_schedule.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">date</t>
   </si>
@@ -53,7 +53,7 @@
     <t xml:space="preserve">keycard_drop_rooms</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: 814, 1713</t>
+    <t xml:space="preserve">Keydrops today: 1713</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 1600</t>
@@ -65,6 +65,9 @@
     <t xml:space="preserve">Keydrops today: 716</t>
   </si>
   <si>
+    <t xml:space="preserve">Keydrops today: 814</t>
+  </si>
+  <si>
     <t xml:space="preserve">Keydrops today: 1615</t>
   </si>
   <si>
@@ -74,10 +77,13 @@
     <t xml:space="preserve">Keydrops today: 513</t>
   </si>
   <si>
-    <t xml:space="preserve">Keydrops today: 1713, 716, 1615</t>
+    <t xml:space="preserve">Keydrops today: 1615, 513</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: 814, 515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keydrops today: 1615, 1600</t>
   </si>
   <si>
     <t xml:space="preserve">Keydrops today: Casa 2-3</t>
@@ -535,7 +541,7 @@
         <v>0</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>13</v>
@@ -730,9 +736,11 @@
         <v>0</v>
       </c>
       <c r="L7" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -772,7 +780,7 @@
         <v>100</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -842,7 +850,7 @@
         <v>400</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
@@ -943,18 +951,28 @@
         <v>100</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
         <v>46094</v>
       </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
+      <c r="B14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G14" s="1" t="n">
         <v>0</v>
       </c>
@@ -962,7 +980,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J14" s="1" t="n">
         <v>0</v>
@@ -971,9 +989,11 @@
         <v>0</v>
       </c>
       <c r="L14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1109,10 +1129,10 @@
         <v>0</v>
       </c>
       <c r="L18" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19">
@@ -1170,7 +1190,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>0</v>
@@ -1191,10 +1211,10 @@
         <v>0</v>
       </c>
       <c r="L20" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21">
@@ -1290,7 +1310,7 @@
         <v>1200</v>
       </c>
       <c r="H23" s="1" t="n">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="I23" s="1" t="n">
         <v>0</v>
@@ -1302,10 +1322,10 @@
         <v>0</v>
       </c>
       <c r="L23" s="1" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="24">
@@ -1331,7 +1351,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I24" s="1" t="n">
         <v>1200</v>
@@ -1343,10 +1363,10 @@
         <v>0</v>
       </c>
       <c r="L24" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25">
@@ -1387,7 +1407,7 @@
         <v>200</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26">
@@ -1415,26 +1435,34 @@
         <v>0</v>
       </c>
       <c r="L26" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="M26" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M26" s="1"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
         <v>46107</v>
       </c>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
+      <c r="B27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G27" s="1" t="n">
         <v>0</v>
       </c>
       <c r="H27" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="I27" s="1" t="n">
         <v>0</v>
@@ -1443,13 +1471,13 @@
         <v>0</v>
       </c>
       <c r="K27" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="L27" s="1" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28">
@@ -1509,18 +1537,28 @@
         <v>100</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
         <v>46110</v>
       </c>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
+      <c r="B30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="1" t="n">
+        <v>0</v>
+      </c>
       <c r="G30" s="1" t="n">
         <v>0</v>
       </c>
@@ -1528,7 +1566,7 @@
         <v>0</v>
       </c>
       <c r="I30" s="1" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J30" s="1" t="n">
         <v>0</v>
@@ -1537,9 +1575,11 @@
         <v>0</v>
       </c>
       <c r="L30" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" s="1"/>
+        <v>100</v>
+      </c>
+      <c r="M30" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1613,7 +1653,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B33" s="3" t="str">
         <f>SUM(B2:F32)</f>

</xml_diff>